<commit_message>
Publica guia ISO/IEC 27090 com licença CC BY-NC 4.0
Remove noindex, adiciona licença e aviso de ausência de garantia,
hospeda fontes localmente (sem chamadas ao Google Fonts no guia),
cria sitemap.xml e robots.txt e adiciona link no menu do portfólio.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ST6Rdqtq9k3Xb3uFmV33DF
</commit_message>
<xml_diff>
--- a/iso27090/modelos/inventario-ia-iso27090.xlsx
+++ b/iso27090/modelos/inventario-ia-iso27090.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="77">
   <si>
     <t xml:space="preserve">Inventário de sistemas de IA · ISO/IEC 27090</t>
   </si>
@@ -49,6 +49,9 @@
   </si>
   <si>
     <t xml:space="preserve">Fonte: guia prático ISO/IEC 27090 em andre0silva.github.io/iso27090. Material de apoio; não reproduz o texto da norma.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Licença: CC BY-NC 4.0 (https://creativecommons.org/licenses/by-nc/4.0/deed.pt-br). © 2026 André Ferreira. Uso livre com crédito ao autor, sem fins comerciais. Fornecido sem garantia.</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -726,7 +729,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -770,6 +773,11 @@
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -813,188 +821,188 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="N2" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="M2" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="N2" s="4" t="s">
-        <v>38</v>
-      </c>
       <c r="O2" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="R2" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="T2" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="R3" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="T3" s="4" t="s">
         <v>45</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="F3" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="R3" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="S3" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="T3" s="4" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5391,100 +5399,100 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>